<commit_message>
cubemx 업데이트, gpio expander 코드 추가
</commit_message>
<xml_diff>
--- a/ID601/Jig/ID601_ES/Docs/Firmware_Development_Documentation.xlsx
+++ b/ID601/Jig/ID601_ES/Docs/Firmware_Development_Documentation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\ID601\Jig\ID601_ES\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B0A5BA-1299-423A-BCEB-D74624BFBCE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B40948F-3891-4EF6-A21C-0ADAA907D8D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" tabRatio="875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Summary" sheetId="14" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="438">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -871,9 +871,6 @@
     <t>CLI Task / Command Parser</t>
   </si>
   <si>
-    <t>FW-REQ-002~005</t>
-  </si>
-  <si>
     <t>UART Driver</t>
   </si>
   <si>
@@ -883,9 +880,6 @@
     <t>USART2, DMA1 Stream6 TX, RX interrupt</t>
   </si>
   <si>
-    <t>FW-REQ-002, 007</t>
-  </si>
-  <si>
     <t>FW-REQ-003~005</t>
   </si>
   <si>
@@ -901,9 +895,6 @@
     <t>Timer Driver</t>
   </si>
   <si>
-    <t>FW-REQ-006, 008</t>
-  </si>
-  <si>
     <t>UART firmware update and application jump</t>
   </si>
   <si>
@@ -934,13 +925,7 @@
     <t>ID804 Core</t>
   </si>
   <si>
-    <t>id804_boot_i2c()</t>
-  </si>
-  <si>
     <t>bool</t>
-  </si>
-  <si>
-    <t>I2C boot topology, power, relay 및 transport를 설정한다.</t>
   </si>
   <si>
     <t>FW-REQ-003, 005</t>
@@ -1428,10 +1413,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>The firmware shall control ID804 through Timer PWM with DMA.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>The firmware shall measure the frequency, current, voltage of ID601 output signal.</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -1456,10 +1437,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>The firmware shall encode ID804 one-wire serial data using timer input capture and CRC-8 SAE J1850.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>ID601 power, relay routing control</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -1504,10 +1481,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Data transfer with SPIx</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>SPI1, SPI2</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -1526,19 +1499,57 @@
     <t>ARC-012</t>
   </si>
   <si>
-    <t>I2C Driver</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Data transfer with I2C</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>I2C1</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>ADC1 IN8</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FW-REQ-009</t>
+  </si>
+  <si>
+    <t>The firmware shall control ID601 through Timer PWM with DMA.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The firmware shall encode ID601 one-wire serial data using timer input capture and CRC-8 SAE J1850.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The firmware shall execute ID601 test or trim sequence.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FW-REQ-009</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The firmware shall generate vsync signal and control LED brightness using ID601.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ARC-013</t>
+  </si>
+  <si>
+    <t>ID601</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>id601_read() / id601_write()</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Data transfer with SPIx to control ADS114S08 (and IC603 if needed)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCP23017 Driver</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCP23017 register read/write using I2C</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1665,7 +1676,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1723,15 +1734,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1739,7 +1741,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1798,6 +1800,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1807,16 +1815,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2221,7 +2220,7 @@
         <v>59</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -2236,16 +2235,16 @@
       <c r="B5" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="25" t="s">
-        <v>404</v>
+      <c r="C5" s="22" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="C6" s="26" t="s">
-        <v>405</v>
+      <c r="C6" s="23" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -2460,7 +2459,7 @@
         <v>70</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>407</v>
+        <v>427</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>9</v>
@@ -2482,7 +2481,7 @@
         <v>70</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>414</v>
+        <v>428</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>9</v>
@@ -2490,6 +2489,7 @@
       <c r="F6" s="4" t="s">
         <v>14</v>
       </c>
+      <c r="G6" s="12"/>
       <c r="H6" s="4" t="s">
         <v>12</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>69</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>9</v>
@@ -2561,8 +2561,50 @@
       </c>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="11" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="10" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B10" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="12"/>
+      <c r="H10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="12"/>
+    </row>
+    <row r="11" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B11" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="12"/>
+      <c r="H11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="12"/>
+    </row>
     <row r="12" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="13" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
@@ -2576,19 +2618,19 @@
           <x14:formula1>
             <xm:f>Common!$D$3:$D$7</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H9</xm:sqref>
+          <xm:sqref>H3:H11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5DF9B7D1-31DB-4402-87DE-866074A4475D}">
           <x14:formula1>
             <xm:f>Common!$B$3:$B$5</xm:f>
           </x14:formula1>
-          <xm:sqref>E3:E9</xm:sqref>
+          <xm:sqref>E3:E11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A450BA07-13EB-4D36-880F-44F80B40A943}">
           <x14:formula1>
             <xm:f>Common!$C$3:$C$4</xm:f>
           </x14:formula1>
-          <xm:sqref>F3:F9</xm:sqref>
+          <xm:sqref>F3:F11</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2674,13 +2716,13 @@
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>242</v>
+        <v>13</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>12</v>
@@ -2695,16 +2737,16 @@
         <v>28</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>8</v>
+        <v>229</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>12</v>
@@ -2719,15 +2761,17 @@
         <v>28</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>422</v>
-      </c>
-      <c r="G6" s="4"/>
+        <v>415</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>426</v>
+      </c>
       <c r="H6" s="5" t="s">
         <v>12</v>
       </c>
@@ -2741,16 +2785,16 @@
         <v>31</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>245</v>
-      </c>
       <c r="G7" s="4" t="s">
-        <v>246</v>
+        <v>13</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>12</v>
@@ -2765,16 +2809,16 @@
         <v>31</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>12</v>
@@ -2789,15 +2833,17 @@
         <v>31</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>425</v>
-      </c>
-      <c r="G9" s="4"/>
+        <v>418</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>229</v>
+      </c>
       <c r="H9" s="5" t="s">
         <v>12</v>
       </c>
@@ -2810,20 +2856,21 @@
       <c r="C10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>419</v>
+      <c r="D10" s="27" t="s">
+        <v>436</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>426</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>427</v>
-      </c>
-      <c r="G10" s="4"/>
+        <v>437</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>424</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>229</v>
+      </c>
       <c r="H10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="5"/>
     </row>
     <row r="11" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="4" t="s">
@@ -2836,10 +2883,10 @@
         <v>412</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>415</v>
+        <v>435</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>250</v>
+        <v>419</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>20</v>
@@ -2851,22 +2898,22 @@
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B12" s="4" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>31</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>251</v>
+        <v>406</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>417</v>
+        <v>248</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>252</v>
+        <v>229</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>12</v>
@@ -2875,41 +2922,55 @@
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B13" s="4" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="27" t="s">
-        <v>429</v>
-      </c>
-      <c r="E13" s="27" t="s">
-        <v>430</v>
-      </c>
-      <c r="F13" s="27" t="s">
-        <v>435</v>
-      </c>
+      <c r="D13" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" s="5"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B14" s="4" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14" s="12"/>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B15" s="4" t="s">
         <v>432</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="F14" s="28" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="4" t="s">
-        <v>431</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>237</v>
@@ -2918,13 +2979,13 @@
         <v>218</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>12</v>
@@ -2932,21 +2993,28 @@
       <c r="I15" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="B2:I15" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I25">
-      <sortCondition descending="1" ref="C2:C15"/>
+  <autoFilter ref="B2:I14" xr:uid="{00000000-0009-0000-0000-000001000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I24">
+      <sortCondition descending="1" ref="C2:C14"/>
     </sortState>
   </autoFilter>
+  <dataConsolidate/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{906586F3-ADBA-48AA-8AFA-20F2BBA23786}">
           <x14:formula1>
             <xm:f>Common!$D$3:$D$7</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H12 H15</xm:sqref>
+          <xm:sqref>H3:H15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{69798CE6-F365-4CCD-A33E-7959614CF98C}">
+          <x14:formula1>
+            <xm:f>'01_Requirement'!$B$3:$B$36</xm:f>
+          </x14:formula1>
+          <xm:sqref>G3:G25</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3008,22 +3076,22 @@
         <v>40</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>258</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>261</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>13</v>
@@ -3037,25 +3105,23 @@
         <v>42</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>262</v>
+        <v>433</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>263</v>
+        <v>434</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>41</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>265</v>
-      </c>
+        <v>260</v>
+      </c>
+      <c r="G4" s="4"/>
       <c r="H4" s="4" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>72</v>
@@ -3066,25 +3132,25 @@
         <v>43</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>267</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="F5" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>269</v>
-      </c>
       <c r="H5" s="4" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>72</v>
@@ -3095,22 +3161,22 @@
         <v>44</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>16</v>
@@ -3121,25 +3187,25 @@
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B7" s="12" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>16</v>
@@ -3150,28 +3216,28 @@
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B8" s="12" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>72</v>
@@ -3179,25 +3245,25 @@
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B9" s="12" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="F9" s="12" t="s">
         <v>41</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>20</v>
@@ -3208,25 +3274,25 @@
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B10" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="G10" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="H10" s="12" t="s">
         <v>291</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>292</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>294</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>295</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>296</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>117</v>
@@ -3237,25 +3303,25 @@
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B11" s="12" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>218</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="I11" s="12" t="s">
         <v>120</v>
@@ -3266,25 +3332,25 @@
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B12" s="12" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>218</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>41</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="I12" s="12" t="s">
         <v>120</v>
@@ -3361,60 +3427,60 @@
         <v>52</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>135</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>224</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B4" s="2" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>224</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.45">
@@ -3425,28 +3491,28 @@
         <v>52</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>224</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.45">
@@ -3457,124 +3523,124 @@
         <v>52</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>224</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B7" s="2" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>224</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="C8" t="s">
         <v>52</v>
       </c>
       <c r="D8" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="E8" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="F8" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="G8" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="H8" t="s">
         <v>224</v>
       </c>
       <c r="I8" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K8" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C9" t="s">
         <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="E9" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="F9" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="G9" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="H9" t="s">
         <v>224</v>
       </c>
       <c r="I9" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="J9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K9" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -3649,19 +3715,19 @@
         <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>224</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>221</v>
@@ -3673,7 +3739,7 @@
         <v>127</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.45">
@@ -3684,19 +3750,19 @@
         <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>224</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>221</v>
@@ -3708,7 +3774,7 @@
         <v>127</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.45">
@@ -3719,19 +3785,19 @@
         <v>16</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>224</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>221</v>
@@ -3743,7 +3809,7 @@
         <v>127</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.45">
@@ -3754,19 +3820,19 @@
         <v>18</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>224</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>221</v>
@@ -3778,7 +3844,7 @@
         <v>127</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.45">
@@ -3789,19 +3855,19 @@
         <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>224</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>221</v>
@@ -3813,7 +3879,7 @@
         <v>127</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.45">
@@ -3824,19 +3890,19 @@
         <v>117</v>
       </c>
       <c r="D8" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="E8" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="F8" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="G8" t="s">
         <v>224</v>
       </c>
       <c r="H8" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I8" t="s">
         <v>221</v>
@@ -3848,30 +3914,30 @@
         <v>127</v>
       </c>
       <c r="L8" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="C9" t="s">
         <v>120</v>
       </c>
       <c r="D9" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="E9" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="F9" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="G9" t="s">
         <v>224</v>
       </c>
       <c r="H9" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I9" t="s">
         <v>221</v>
@@ -3883,30 +3949,30 @@
         <v>127</v>
       </c>
       <c r="L9" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="C10" t="s">
         <v>120</v>
       </c>
       <c r="D10" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="E10" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="F10" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="G10" t="s">
         <v>224</v>
       </c>
       <c r="H10" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I10" t="s">
         <v>221</v>
@@ -3918,7 +3984,7 @@
         <v>127</v>
       </c>
       <c r="L10" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.45">
@@ -3929,19 +3995,19 @@
         <v>229</v>
       </c>
       <c r="D11" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E11" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="F11" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="G11" t="s">
         <v>224</v>
       </c>
       <c r="H11" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I11" t="s">
         <v>221</v>
@@ -3953,7 +4019,7 @@
         <v>127</v>
       </c>
       <c r="L11" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -3992,10 +4058,10 @@
       <c r="D2" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="F2" s="24"/>
+      <c r="F2" s="26"/>
       <c r="G2" s="14" t="s">
         <v>125</v>
       </c>
@@ -4103,80 +4169,80 @@
       <c r="G8" s="15"/>
     </row>
     <row r="9" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="24" t="s">
         <v>143</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="24" t="s">
         <v>144</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="G9" s="22"/>
+      <c r="G9" s="24"/>
     </row>
     <row r="10" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="22"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="22"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="24"/>
     </row>
     <row r="11" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="22"/>
+      <c r="B11" s="24"/>
       <c r="C11" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="22"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="24"/>
     </row>
     <row r="12" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="24" t="s">
         <v>145</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="F12" s="23" t="s">
+      <c r="F12" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="G12" s="22"/>
+      <c r="G12" s="24"/>
     </row>
     <row r="13" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="22"/>
+      <c r="B13" s="24"/>
       <c r="C13" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="22"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="24"/>
     </row>
     <row r="14" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="22"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="22"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="24"/>
     </row>
     <row r="15" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B15" s="15" t="s">
@@ -4347,13 +4413,13 @@
       <c r="G23" s="15"/>
     </row>
     <row r="24" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="24" t="s">
         <v>205</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="24" t="s">
         <v>196</v>
       </c>
       <c r="E24" s="15" t="s">
@@ -4362,30 +4428,30 @@
       <c r="F24" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="G24" s="22" t="s">
+      <c r="G24" s="24" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
       <c r="E25" s="15" t="s">
         <v>207</v>
       </c>
       <c r="F25" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="G25" s="22"/>
+      <c r="G25" s="24"/>
     </row>
     <row r="26" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="24" t="s">
         <v>208</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="D26" s="24" t="s">
         <v>165</v>
       </c>
       <c r="E26" s="15" t="s">
@@ -4394,21 +4460,21 @@
       <c r="F26" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="G26" s="22" t="s">
+      <c r="G26" s="24" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
       <c r="E27" s="15" t="s">
         <v>210</v>
       </c>
       <c r="F27" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="G27" s="22"/>
+      <c r="G27" s="24"/>
     </row>
     <row r="28" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="29" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -4462,7 +4528,7 @@
         <v>84</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.45">
@@ -4636,24 +4702,24 @@
         <v>93</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="D9" s="11" t="s">
+        <v>392</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>395</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="G9" s="11" t="s">
         <v>397</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>400</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>401</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>402</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
       <c r="J9" s="11" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="K9" s="11"/>
       <c r="L9" s="11"/>
@@ -5162,15 +5228,15 @@
         <v>67</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B3" s="2" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="D3" t="s">
         <v>61</v>
@@ -5179,7 +5245,7 @@
         <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="G3" s="21">
         <v>46281</v>
@@ -5188,10 +5254,10 @@
         <v>46281</v>
       </c>
       <c r="I3" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="J3" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.45">

</xml_diff>